<commit_message>
rcaplaybook edit and internalID for incidentkey
</commit_message>
<xml_diff>
--- a/soldoc/npe-incident-traiging-solution-deliveryv0.1.xlsx
+++ b/soldoc/npe-incident-traiging-solution-deliveryv0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SourceCode\non-prod-incident-triaging\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\gitdir\AgenticAI_DIR\npe-incidents-triaging-rca\soldoc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{454F0A88-C2E6-4E87-A776-7186DF78656F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C3376E2-7E8D-4974-B62D-42269B099EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="3" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2235" yWindow="1785" windowWidth="21600" windowHeight="11160" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E2E Solution" sheetId="7" r:id="rId1"/>
@@ -2791,9 +2791,6 @@
     </r>
   </si>
   <si>
-    <t>Executes approved playbooks — ordered checks, retries, continue-on-error.</t>
-  </si>
-  <si>
     <t>Diagnostic checks</t>
   </si>
   <si>
@@ -3217,6 +3214,10 @@
   </si>
   <si>
     <t>Planned — API is trusted-network-only today; MSAL elsewhere in the stack only covers the Teams Graph poller, a separate trust boundary</t>
+  </si>
+  <si>
+    <t>Executes approved playbooks — ordered checks, retries, continue-on-error.
+https://github.com/open-workflow-specification/specification/blob/main/dsl-reference.md</t>
   </si>
 </sst>
 </file>
@@ -3713,9 +3714,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3753,7 +3754,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3859,7 +3860,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4001,7 +4002,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4010,11 +4011,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D853524-532F-43BC-A398-76BE74ABF484}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="35"/>
+    <col min="1" max="1" width="9.109375" style="35"/>
     <col min="2" max="2" width="27" style="39" customWidth="1"/>
-    <col min="3" max="3" width="155.85546875" style="39" customWidth="1"/>
+    <col min="3" max="3" width="155.88671875" style="39" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4039,7 +4040,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="45.75">
+    <row r="3" spans="1:3" ht="43.2">
       <c r="A3" s="34" t="s">
         <v>6</v>
       </c>
@@ -4105,7 +4106,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="45.75">
+    <row r="9" spans="1:3" ht="43.2">
       <c r="A9" s="34" t="s">
         <v>24</v>
       </c>
@@ -4126,16 +4127,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEC7BCEF-5B70-475C-B97D-11685B3F008F}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4.85546875" customWidth="1"/>
-    <col min="2" max="2" width="29.7109375" customWidth="1"/>
-    <col min="3" max="3" width="124.5703125" customWidth="1"/>
-    <col min="4" max="4" width="125.28515625" customWidth="1"/>
-    <col min="5" max="5" width="49.85546875" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="124.5546875" customWidth="1"/>
+    <col min="4" max="4" width="125.33203125" customWidth="1"/>
+    <col min="5" max="5" width="49.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="39" customFormat="1" ht="17.25">
+    <row r="1" spans="1:4" s="39" customFormat="1" ht="15.6">
       <c r="A1" s="41" t="s">
         <v>27</v>
       </c>
@@ -4149,7 +4150,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="2" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A2" s="43">
         <v>1</v>
       </c>
@@ -4163,7 +4164,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="3" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A3" s="43">
         <v>2</v>
       </c>
@@ -4177,7 +4178,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="4" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A4" s="43">
         <v>3</v>
       </c>
@@ -4191,7 +4192,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="5" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A5" s="43">
         <v>4</v>
       </c>
@@ -4205,7 +4206,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="39" customFormat="1" ht="17.25">
+    <row r="6" spans="1:4" s="39" customFormat="1" ht="15.6">
       <c r="A6" s="43">
         <v>5</v>
       </c>
@@ -4219,7 +4220,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="7" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A7" s="43">
         <v>6</v>
       </c>
@@ -4233,7 +4234,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="8" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A8" s="43">
         <v>7</v>
       </c>
@@ -4247,7 +4248,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="9" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A9" s="43">
         <v>8</v>
       </c>
@@ -4261,7 +4262,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="10" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A10" s="43">
         <v>9</v>
       </c>
@@ -4275,7 +4276,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="11" spans="1:4" s="39" customFormat="1" ht="15.6">
       <c r="A11" s="43">
         <v>10</v>
       </c>
@@ -4289,7 +4290,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="12" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A12" s="43">
         <v>11</v>
       </c>
@@ -4303,7 +4304,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="39" customFormat="1" ht="36">
+    <row r="13" spans="1:4" s="39" customFormat="1" ht="30">
       <c r="A13" s="43">
         <v>12</v>
       </c>
@@ -4325,7 +4326,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78A2922D-DECF-4840-9467-9B2ED21F406F}">
   <dimension ref="AA11"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="11" spans="27:27">
       <c r="AA11" t="s">
@@ -4343,12 +4344,12 @@
   <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="18" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="2" width="28.140625" customWidth="1"/>
-    <col min="3" max="3" width="68.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.42578125" customWidth="1"/>
-    <col min="5" max="5" width="64.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26.42578125" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" customWidth="1"/>
+    <col min="2" max="2" width="28.109375" customWidth="1"/>
+    <col min="3" max="3" width="68.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" customWidth="1"/>
+    <col min="5" max="5" width="64.6640625" customWidth="1"/>
+    <col min="6" max="6" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1">
@@ -4371,7 +4372,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="8" customFormat="1" ht="32.450000000000003" customHeight="1">
+    <row r="2" spans="1:6" s="8" customFormat="1" ht="32.4" customHeight="1">
       <c r="A2" s="12">
         <v>1</v>
       </c>
@@ -4461,7 +4462,7 @@
       </c>
       <c r="F6" s="7"/>
     </row>
-    <row r="7" spans="1:6" s="8" customFormat="1" ht="37.9" customHeight="1">
+    <row r="7" spans="1:6" s="8" customFormat="1" ht="37.950000000000003" customHeight="1">
       <c r="A7" s="12">
         <v>6</v>
       </c>
@@ -4479,7 +4480,7 @@
       </c>
       <c r="F7" s="7"/>
     </row>
-    <row r="8" spans="1:6" s="8" customFormat="1" ht="25.15" customHeight="1">
+    <row r="8" spans="1:6" s="8" customFormat="1" ht="25.2" customHeight="1">
       <c r="A8" s="12">
         <v>7</v>
       </c>
@@ -4515,7 +4516,7 @@
       </c>
       <c r="F9" s="7"/>
     </row>
-    <row r="10" spans="1:6" s="8" customFormat="1" ht="20.45" customHeight="1">
+    <row r="10" spans="1:6" s="8" customFormat="1" ht="20.399999999999999" customHeight="1">
       <c r="A10" s="12">
         <v>9</v>
       </c>
@@ -4551,7 +4552,7 @@
       </c>
       <c r="F11" s="7"/>
     </row>
-    <row r="12" spans="1:6" ht="32.450000000000003" customHeight="1">
+    <row r="12" spans="1:6" ht="32.4" customHeight="1">
       <c r="A12" s="12">
         <v>11</v>
       </c>
@@ -4569,7 +4570,7 @@
       </c>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:6" ht="32.450000000000003" customHeight="1">
+    <row r="13" spans="1:6" ht="32.4" customHeight="1">
       <c r="A13" s="12">
         <v>12</v>
       </c>
@@ -4587,7 +4588,7 @@
       </c>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" spans="1:6" ht="46.15" customHeight="1">
+    <row r="14" spans="1:6" ht="46.2" customHeight="1">
       <c r="A14" s="12">
         <v>13</v>
       </c>
@@ -4623,7 +4624,7 @@
       </c>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" spans="1:6" ht="20.45" customHeight="1">
+    <row r="16" spans="1:6" ht="20.399999999999999" customHeight="1">
       <c r="A16" s="12">
         <v>15</v>
       </c>
@@ -4641,7 +4642,7 @@
       </c>
       <c r="F16" s="3"/>
     </row>
-    <row r="17" spans="1:6" ht="34.9" customHeight="1">
+    <row r="17" spans="1:6" ht="34.950000000000003" customHeight="1">
       <c r="A17" s="12">
         <v>16</v>
       </c>
@@ -4738,20 +4739,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8729759-D495-4EF8-9594-03671ED760C0}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="40.9" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="40.950000000000003" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" style="13" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" style="13" customWidth="1"/>
-    <col min="3" max="3" width="30.5703125" style="13" customWidth="1"/>
-    <col min="4" max="4" width="52.7109375" style="13" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="13" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="13" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" style="13" customWidth="1"/>
-    <col min="8" max="8" width="33.5703125" style="13" customWidth="1"/>
-    <col min="9" max="16384" width="8.85546875" style="13"/>
+    <col min="1" max="1" width="4.6640625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" style="13" customWidth="1"/>
+    <col min="3" max="3" width="30.5546875" style="13" customWidth="1"/>
+    <col min="4" max="4" width="52.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="13" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" style="13" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" style="13" customWidth="1"/>
+    <col min="8" max="8" width="33.5546875" style="13" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="40.9" customHeight="1">
+    <row r="1" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A1" s="14" t="s">
         <v>27</v>
       </c>
@@ -4777,7 +4778,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="40.9" customHeight="1">
+    <row r="2" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A2" s="16">
         <v>1</v>
       </c>
@@ -4825,7 +4826,7 @@
       </c>
       <c r="H3" s="22"/>
     </row>
-    <row r="4" spans="1:8" ht="40.9" customHeight="1">
+    <row r="4" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A4" s="16">
         <v>3</v>
       </c>
@@ -4849,7 +4850,7 @@
       </c>
       <c r="H4" s="22"/>
     </row>
-    <row r="5" spans="1:8" ht="40.9" customHeight="1">
+    <row r="5" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A5" s="16">
         <v>4</v>
       </c>
@@ -4873,7 +4874,7 @@
       </c>
       <c r="H5" s="22"/>
     </row>
-    <row r="6" spans="1:8" ht="40.9" customHeight="1">
+    <row r="6" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A6" s="16">
         <v>5</v>
       </c>
@@ -4897,7 +4898,7 @@
       </c>
       <c r="H6" s="22"/>
     </row>
-    <row r="7" spans="1:8" ht="40.9" customHeight="1">
+    <row r="7" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A7" s="16">
         <v>6</v>
       </c>
@@ -4921,11 +4922,11 @@
       </c>
       <c r="H7" s="22"/>
     </row>
-    <row r="8" spans="1:8" ht="40.9" customHeight="1">
+    <row r="8" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="G8" s="27"/>
       <c r="H8" s="22"/>
     </row>
-    <row r="9" spans="1:8" ht="40.9" customHeight="1">
+    <row r="9" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A9" s="19">
         <v>7</v>
       </c>
@@ -4997,7 +4998,7 @@
       </c>
       <c r="H11" s="22"/>
     </row>
-    <row r="12" spans="1:8" ht="40.9" customHeight="1">
+    <row r="12" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A12" s="19">
         <v>10</v>
       </c>
@@ -5021,7 +5022,7 @@
       </c>
       <c r="H12" s="22"/>
     </row>
-    <row r="13" spans="1:8" ht="40.9" customHeight="1">
+    <row r="13" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A13" s="19">
         <v>11</v>
       </c>
@@ -5045,7 +5046,7 @@
       </c>
       <c r="H13" s="22"/>
     </row>
-    <row r="14" spans="1:8" ht="40.9" customHeight="1">
+    <row r="14" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A14" s="19">
         <v>12</v>
       </c>
@@ -5069,7 +5070,7 @@
       </c>
       <c r="H14" s="22"/>
     </row>
-    <row r="15" spans="1:8" ht="40.9" customHeight="1">
+    <row r="15" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A15" s="19">
         <v>13</v>
       </c>
@@ -5093,7 +5094,7 @@
       </c>
       <c r="H15" s="22"/>
     </row>
-    <row r="16" spans="1:8" ht="40.9" customHeight="1">
+    <row r="16" spans="1:8" ht="40.950000000000003" customHeight="1">
       <c r="A16" s="19">
         <v>14</v>
       </c>
@@ -5125,15 +5126,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F731AFB6-5CB8-403D-9EC1-A8BA71F57706}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
-    <col min="3" max="3" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.109375" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" customWidth="1"/>
     <col min="4" max="4" width="98" customWidth="1"/>
-    <col min="5" max="5" width="85.140625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="85.109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.25">
+    <row r="1" spans="1:5" ht="15.6">
       <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
@@ -5150,7 +5151,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17.25">
+    <row r="2" spans="1:5" ht="15.6">
       <c r="A2" s="31">
         <v>1</v>
       </c>
@@ -5167,7 +5168,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="36">
+    <row r="3" spans="1:5" ht="30.6">
       <c r="A3" s="29">
         <v>2</v>
       </c>
@@ -5184,7 +5185,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="36">
+    <row r="4" spans="1:5" ht="30.6">
       <c r="A4" s="29">
         <v>3</v>
       </c>
@@ -5201,7 +5202,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="36">
+    <row r="5" spans="1:5" ht="30.6">
       <c r="A5" s="29">
         <v>4</v>
       </c>
@@ -5218,7 +5219,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="36">
+    <row r="6" spans="1:5" ht="30.6">
       <c r="A6" s="29">
         <v>5</v>
       </c>
@@ -5235,7 +5236,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="53.25">
+    <row r="7" spans="1:5" ht="30.6">
       <c r="A7" s="29">
         <v>6</v>
       </c>
@@ -5252,7 +5253,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="17.25">
+    <row r="8" spans="1:5" ht="15.6">
       <c r="A8" s="29">
         <v>7</v>
       </c>
@@ -5269,7 +5270,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="36">
+    <row r="9" spans="1:5" ht="30.6">
       <c r="A9" s="29">
         <v>8</v>
       </c>
@@ -5286,7 +5287,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="36">
+    <row r="10" spans="1:5" ht="30.6">
       <c r="A10" s="29">
         <v>9</v>
       </c>
@@ -5303,7 +5304,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="53.25">
+    <row r="11" spans="1:5" ht="45.6">
       <c r="A11" s="29">
         <v>10</v>
       </c>
@@ -5314,214 +5315,214 @@
         <v>212</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>213</v>
+        <v>255</v>
       </c>
       <c r="E11" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="124.5">
+    <row r="12" spans="1:5" ht="90.6">
       <c r="A12" s="29">
         <v>11</v>
       </c>
       <c r="B12" s="29" t="s">
+        <v>213</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>214</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="D12" s="29" t="s">
         <v>215</v>
       </c>
-      <c r="D12" s="29" t="s">
+      <c r="E12" s="28" t="s">
         <v>216</v>
       </c>
-      <c r="E12" s="28" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="53.25">
+    </row>
+    <row r="13" spans="1:5" ht="45.6">
       <c r="A13" s="29">
         <v>12</v>
       </c>
       <c r="B13" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="29" t="s">
         <v>218</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="D13" s="29" t="s">
         <v>219</v>
-      </c>
-      <c r="D13" s="29" t="s">
-        <v>220</v>
       </c>
       <c r="E13" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="36">
+    <row r="14" spans="1:5" ht="30.6">
       <c r="A14" s="29">
         <v>13</v>
       </c>
       <c r="B14" s="29" t="s">
+        <v>220</v>
+      </c>
+      <c r="C14" s="29" t="s">
         <v>221</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="D14" s="29" t="s">
         <v>222</v>
-      </c>
-      <c r="D14" s="29" t="s">
-        <v>223</v>
       </c>
       <c r="E14" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="17.25">
+    <row r="15" spans="1:5" ht="15.6">
       <c r="A15" s="29">
         <v>14</v>
       </c>
       <c r="B15" s="29" t="s">
+        <v>223</v>
+      </c>
+      <c r="C15" s="29" t="s">
         <v>224</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="D15" s="29" t="s">
         <v>225</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>226</v>
       </c>
       <c r="E15" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="17.25">
+    <row r="16" spans="1:5" ht="15.6">
       <c r="A16" s="29">
         <v>15</v>
       </c>
       <c r="B16" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="C16" s="29" t="s">
         <v>227</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="D16" s="29" t="s">
         <v>228</v>
       </c>
-      <c r="D16" s="29" t="s">
+      <c r="E16" s="29" t="s">
         <v>229</v>
       </c>
-      <c r="E16" s="29" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="36">
+    </row>
+    <row r="17" spans="1:5" ht="30.6">
       <c r="A17" s="29">
         <v>16</v>
       </c>
       <c r="B17" s="29" t="s">
+        <v>230</v>
+      </c>
+      <c r="C17" s="29" t="s">
         <v>231</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="D17" s="29" t="s">
         <v>232</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>233</v>
       </c>
       <c r="E17" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="36">
+    <row r="18" spans="1:5" ht="30.6">
       <c r="A18" s="29">
         <v>17</v>
       </c>
       <c r="B18" s="29" t="s">
+        <v>233</v>
+      </c>
+      <c r="C18" s="29" t="s">
         <v>234</v>
       </c>
-      <c r="C18" s="29" t="s">
+      <c r="D18" s="29" t="s">
         <v>235</v>
-      </c>
-      <c r="D18" s="29" t="s">
-        <v>236</v>
       </c>
       <c r="E18" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="53.25">
+    <row r="19" spans="1:5" ht="45.6">
       <c r="A19" s="29">
         <v>18</v>
       </c>
       <c r="B19" s="29" t="s">
+        <v>236</v>
+      </c>
+      <c r="C19" s="29" t="s">
         <v>237</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="D19" s="29" t="s">
         <v>238</v>
       </c>
-      <c r="D19" s="29" t="s">
+      <c r="E19" s="29" t="s">
         <v>239</v>
       </c>
-      <c r="E19" s="29" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="36">
+    </row>
+    <row r="20" spans="1:5" ht="31.2">
       <c r="A20" s="29">
         <v>19</v>
       </c>
       <c r="B20" s="29" t="s">
+        <v>240</v>
+      </c>
+      <c r="C20" s="29" t="s">
         <v>241</v>
       </c>
-      <c r="C20" s="29" t="s">
+      <c r="D20" s="29" t="s">
         <v>242</v>
       </c>
-      <c r="D20" s="29" t="s">
+      <c r="E20" s="28" t="s">
         <v>243</v>
       </c>
-      <c r="E20" s="28" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="36">
+    </row>
+    <row r="21" spans="1:5" ht="30.6">
       <c r="A21" s="29">
         <v>20</v>
       </c>
       <c r="B21" s="29" t="s">
+        <v>244</v>
+      </c>
+      <c r="C21" s="29" t="s">
         <v>245</v>
       </c>
-      <c r="C21" s="29" t="s">
+      <c r="D21" s="29" t="s">
         <v>246</v>
       </c>
-      <c r="D21" s="29" t="s">
+      <c r="E21" s="29" t="s">
         <v>247</v>
       </c>
-      <c r="E21" s="29" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="17.25">
+    </row>
+    <row r="22" spans="1:5" ht="15.6">
       <c r="A22" s="29">
         <v>21</v>
       </c>
       <c r="B22" s="29" t="s">
+        <v>248</v>
+      </c>
+      <c r="C22" s="29" t="s">
         <v>249</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="D22" s="29" t="s">
         <v>250</v>
       </c>
-      <c r="D22" s="29" t="s">
+      <c r="E22" s="29" t="s">
         <v>251</v>
       </c>
-      <c r="E22" s="29" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="36">
+    </row>
+    <row r="23" spans="1:5" ht="30.6">
       <c r="A23" s="29">
         <v>22</v>
       </c>
       <c r="B23" s="29" t="s">
+        <v>252</v>
+      </c>
+      <c r="C23" s="29" t="s">
+        <v>241</v>
+      </c>
+      <c r="D23" s="29" t="s">
         <v>253</v>
       </c>
-      <c r="C23" s="29" t="s">
-        <v>242</v>
-      </c>
-      <c r="D23" s="29" t="s">
+      <c r="E23" s="29" t="s">
         <v>254</v>
-      </c>
-      <c r="E23" s="29" t="s">
-        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>